<commit_message>
Refine v3 quiz prompts and attempt tokens
</commit_message>
<xml_diff>
--- a/v3/CS0006/CS0006_DevSpec.xlsx
+++ b/v3/CS0006/CS0006_DevSpec.xlsx
@@ -1197,17 +1197,17 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>SC18</t>
+          <t>SC09</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>CS0006_SC18_I.webp</t>
+          <t>CS0006_SC09_I.webp</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>SC18</t>
+          <t>SC09</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr"/>
@@ -1663,7 +1663,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>mouse.</t>
+          <t>a stone.</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
@@ -1683,7 +1683,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>the</t>
+          <t>under</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
@@ -1703,7 +1703,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>on</t>
+          <t>clothes</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
@@ -1723,7 +1723,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>jumped</t>
+          <t>his</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
@@ -1743,7 +1743,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Cat</t>
+          <t>hid</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
@@ -1763,7 +1763,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>The</t>
+          <t>The Cat</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr"/>
@@ -2414,7 +2414,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>The</t>
+          <t>The Cat</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -2443,7 +2443,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Cat</t>
+          <t>hid</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -2472,7 +2472,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>jumped</t>
+          <t>his</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -2501,7 +2501,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>on</t>
+          <t>clothes</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -2530,7 +2530,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>the</t>
+          <t>under</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -2559,7 +2559,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>mouse.</t>
+          <t>a stone.</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">

</xml_diff>